<commit_message>
completed project, with API and Front end
</commit_message>
<xml_diff>
--- a/new_data_loan.csv.xlsx
+++ b/new_data_loan.csv.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IITK\Projects\Learning_repo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8B637BF-2FBD-4CF8-9BD3-099DD5BD3DB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{730A968C-C7C7-44D6-BB99-0B6A50450B25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{90F78128-A63D-47AD-8B5F-46F246C5472C}"/>
   </bookViews>
@@ -434,10 +434,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6DC35A0-AF14-49E3-A14E-93BE7FF88389}">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1">
         <v>477</v>
       </c>
@@ -474,8 +474,11 @@
       <c r="L1">
         <v>2</v>
       </c>
+      <c r="M1">
+        <v>0</v>
+      </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>478</v>
       </c>
@@ -512,8 +515,11 @@
       <c r="L2">
         <v>3</v>
       </c>
+      <c r="M2">
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>479</v>
       </c>
@@ -550,8 +556,11 @@
       <c r="L3">
         <v>3</v>
       </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>480</v>
       </c>
@@ -588,8 +597,11 @@
       <c r="L4">
         <v>2</v>
       </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>481</v>
       </c>
@@ -625,6 +637,9 @@
       </c>
       <c r="L5">
         <v>4</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>